<commit_message>
premiere version géographique fonctionnelle
</commit_message>
<xml_diff>
--- a/input/geo_list_of_nodes - Excel.xlsx
+++ b/input/geo_list_of_nodes - Excel.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x15 xr xr6 xr10">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26731"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\boissieremat\Documents\GitHub\antares-brinkerink-2015\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:40009_{56A303A1-EC40-4F72-91BC-A8706C46E9B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6994059F-C135-4410-B05F-C7282D6BFE7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="25440" windowHeight="15390"/>
+    <workbookView xWindow="-25320" yWindow="-60" windowWidth="25440" windowHeight="15390" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="geo_list_of_nodes" sheetId="2" r:id="rId1"/>
@@ -23,15 +23,15 @@
 </file>
 
 <file path=xl/connections.xml><?xml version="1.0" encoding="utf-8"?>
-<connections xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <connection id="1" keepAlive="1" name="Requête - geo_list_of_nodes - Excel" description="Connexion à la requête « geo_list_of_nodes - Excel » dans le classeur." type="5" refreshedVersion="8" background="1" saveData="1">
+<connections xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16">
+  <connection id="1" xr16:uid="{00000000-0015-0000-FFFF-FFFF00000000}" keepAlive="1" name="Requête - geo_list_of_nodes - Excel" description="Connexion à la requête « geo_list_of_nodes - Excel » dans le classeur." type="5" refreshedVersion="8" background="1" saveData="1">
     <dbPr connection="Provider=Microsoft.Mashup.OleDb.1;Data Source=$Workbook$;Location=&quot;geo_list_of_nodes - Excel&quot;;Extended Properties=&quot;&quot;" command="SELECT * FROM [geo_list_of_nodes - Excel]"/>
   </connection>
 </connections>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1769" uniqueCount="875">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1769" uniqueCount="941">
   <si>
     <t>Node</t>
   </si>
@@ -2052,12 +2052,6 @@
     <t>Alaska</t>
   </si>
   <si>
-    <t>45.6875333395</t>
-  </si>
-  <si>
-    <t>-112.494333916</t>
-  </si>
-  <si>
     <t>NA-USA-AZ</t>
   </si>
   <si>
@@ -2656,12 +2650,216 @@
   </si>
   <si>
     <t>-106.141224</t>
+  </si>
+  <si>
+    <t>64.4459613</t>
+  </si>
+  <si>
+    <t>-149.680909</t>
+  </si>
+  <si>
+    <t>34.395342</t>
+  </si>
+  <si>
+    <t>-111.763275</t>
+  </si>
+  <si>
+    <t>OSM "Arizona"</t>
+  </si>
+  <si>
+    <t>36.7014631</t>
+  </si>
+  <si>
+    <t>-118.755997</t>
+  </si>
+  <si>
+    <t>OSM "California"</t>
+  </si>
+  <si>
+    <t>31.2638905</t>
+  </si>
+  <si>
+    <t>-98.5456116</t>
+  </si>
+  <si>
+    <t>OSM "Texas"</t>
+  </si>
+  <si>
+    <t>27.7567667</t>
+  </si>
+  <si>
+    <t>-81.4639835</t>
+  </si>
+  <si>
+    <t>OSM "Florida"</t>
+  </si>
+  <si>
+    <t>13.45011745</t>
+  </si>
+  <si>
+    <t>144.7577087765826</t>
+  </si>
+  <si>
+    <t>19.593801499999998</t>
+  </si>
+  <si>
+    <t>-155.42837009716908</t>
+  </si>
+  <si>
+    <t>44.4308975</t>
+  </si>
+  <si>
+    <t>-89.6884637</t>
+  </si>
+  <si>
+    <t>OSM "Wisconsin"</t>
+  </si>
+  <si>
+    <t>47.6201461</t>
+  </si>
+  <si>
+    <t>-100.540737</t>
+  </si>
+  <si>
+    <t>OSM "North Dakota"</t>
+  </si>
+  <si>
+    <t>43.4849133</t>
+  </si>
+  <si>
+    <t>-71.6553992</t>
+  </si>
+  <si>
+    <t>OSM "New Hampshire"</t>
+  </si>
+  <si>
+    <t>43.6447642</t>
+  </si>
+  <si>
+    <t>-114.015407</t>
+  </si>
+  <si>
+    <t>OSM "Idaho"</t>
+  </si>
+  <si>
+    <t>43.1561681</t>
+  </si>
+  <si>
+    <t>-75.8449946</t>
+  </si>
+  <si>
+    <t>OSM "New York State"</t>
+  </si>
+  <si>
+    <t>18.2247706</t>
+  </si>
+  <si>
+    <t>-66.4858295</t>
+  </si>
+  <si>
+    <t>38.7251776</t>
+  </si>
+  <si>
+    <t>-105.607716</t>
+  </si>
+  <si>
+    <t>OSM "Colorado"</t>
+  </si>
+  <si>
+    <t>40.9699889</t>
+  </si>
+  <si>
+    <t>-77.7278831</t>
+  </si>
+  <si>
+    <t>OSM "Pennsylvania"</t>
+  </si>
+  <si>
+    <t>43.6211955</t>
+  </si>
+  <si>
+    <t>-84.6824346</t>
+  </si>
+  <si>
+    <t>OSM "Michigan"</t>
+  </si>
+  <si>
+    <t>40.2253569</t>
+  </si>
+  <si>
+    <t>-82.6881395</t>
+  </si>
+  <si>
+    <t>OSM "Ohio"</t>
+  </si>
+  <si>
+    <t>35.2048883</t>
+  </si>
+  <si>
+    <t>-92.4479108</t>
+  </si>
+  <si>
+    <t>OSM "Arkansas"</t>
+  </si>
+  <si>
+    <t>35.7730076</t>
+  </si>
+  <si>
+    <t>-86.2820081</t>
+  </si>
+  <si>
+    <t>OSM "Tennessee"</t>
+  </si>
+  <si>
+    <t>33.2588817</t>
+  </si>
+  <si>
+    <t>-86.8295337</t>
+  </si>
+  <si>
+    <t>OSM "Alabama"</t>
+  </si>
+  <si>
+    <t>38.27312</t>
+  </si>
+  <si>
+    <t>-98.5821872</t>
+  </si>
+  <si>
+    <t>OSM "Kansas"</t>
+  </si>
+  <si>
+    <t>34.9550817</t>
+  </si>
+  <si>
+    <t>-97.2684063</t>
+  </si>
+  <si>
+    <t>OSM "Oklahoma"</t>
+  </si>
+  <si>
+    <t>35.6729639</t>
+  </si>
+  <si>
+    <t>-79.0392919</t>
+  </si>
+  <si>
+    <t>OSM "North Carolina"</t>
+  </si>
+  <si>
+    <t>38.7604815</t>
+  </si>
+  <si>
+    <t>-92.5617875</t>
+  </si>
+  <si>
+    <t>OSM "Missouri"</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -3190,10 +3388,10 @@
   </cellStyles>
   <dxfs count="8">
     <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
+      <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
@@ -3226,12 +3424,8 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/queryTables/queryTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="DonnéesExternes_1" connectionId="1" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0">
+<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="DonnéesExternes_1" connectionId="1" xr16:uid="{00000000-0016-0000-0000-000000000000}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0">
   <queryTableRefresh nextId="8">
     <queryTableFields count="7">
       <queryTableField id="1" name="Column1" tableColumnId="1"/>
@@ -3247,16 +3441,16 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="geo_list_of_nodes___Excel" displayName="geo_list_of_nodes___Excel" ref="A1:G259" tableType="queryTable" totalsRowShown="0" headerRowDxfId="4">
-  <autoFilter ref="A1:G259"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="geo_list_of_nodes___Excel" displayName="geo_list_of_nodes___Excel" ref="A1:G259" tableType="queryTable" totalsRowShown="0" headerRowDxfId="7">
+  <autoFilter ref="A1:G259" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="7">
-    <tableColumn id="1" uniqueName="1" name="Node" queryTableFieldId="1" dataDxfId="7"/>
-    <tableColumn id="2" uniqueName="2" name="Continent" queryTableFieldId="2" dataDxfId="6"/>
-    <tableColumn id="3" uniqueName="3" name="Country" queryTableFieldId="3" dataDxfId="5"/>
-    <tableColumn id="4" uniqueName="4" name="Geographical region" queryTableFieldId="4" dataDxfId="3"/>
-    <tableColumn id="5" uniqueName="5" name="lat" queryTableFieldId="5" dataDxfId="2"/>
-    <tableColumn id="6" uniqueName="6" name="lon" queryTableFieldId="6" dataDxfId="0"/>
-    <tableColumn id="7" uniqueName="7" name="coordinates_source" queryTableFieldId="7" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" uniqueName="1" name="Node" queryTableFieldId="1" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" uniqueName="2" name="Continent" queryTableFieldId="2" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" uniqueName="3" name="Country" queryTableFieldId="3" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" uniqueName="4" name="Geographical region" queryTableFieldId="4" dataDxfId="3"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" uniqueName="5" name="lat" queryTableFieldId="5" dataDxfId="2"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" uniqueName="6" name="lon" queryTableFieldId="6" dataDxfId="1"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" uniqueName="7" name="coordinates_source" queryTableFieldId="7" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3558,20 +3752,20 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G259"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.7265625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.1796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.54296875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="33.6328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.08984375" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18.453125" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="35.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3582,7 +3776,7 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>810</v>
+        <v>808</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>3</v>
@@ -3594,7 +3788,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
@@ -3617,7 +3811,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>11</v>
       </c>
@@ -3640,7 +3834,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>13</v>
       </c>
@@ -3663,7 +3857,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>17</v>
       </c>
@@ -3686,7 +3880,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>21</v>
       </c>
@@ -3709,7 +3903,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>25</v>
       </c>
@@ -3732,7 +3926,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>29</v>
       </c>
@@ -3755,7 +3949,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>32</v>
       </c>
@@ -3778,7 +3972,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>36</v>
       </c>
@@ -3801,7 +3995,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>38</v>
       </c>
@@ -3824,7 +4018,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>40</v>
       </c>
@@ -3847,7 +4041,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>44</v>
       </c>
@@ -3870,7 +4064,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>48</v>
       </c>
@@ -3893,7 +4087,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>52</v>
       </c>
@@ -3916,7 +4110,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>56</v>
       </c>
@@ -3939,7 +4133,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>60</v>
       </c>
@@ -3959,10 +4153,10 @@
         <v>-13.892143024999999</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>811</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>62</v>
       </c>
@@ -3985,7 +4179,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>66</v>
       </c>
@@ -4008,7 +4202,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>70</v>
       </c>
@@ -4031,7 +4225,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>74</v>
       </c>
@@ -4054,7 +4248,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>78</v>
       </c>
@@ -4077,7 +4271,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>82</v>
       </c>
@@ -4100,7 +4294,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>86</v>
       </c>
@@ -4123,7 +4317,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>90</v>
       </c>
@@ -4146,7 +4340,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>94</v>
       </c>
@@ -4169,7 +4363,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>98</v>
       </c>
@@ -4192,7 +4386,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>100</v>
       </c>
@@ -4215,7 +4409,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>104</v>
       </c>
@@ -4238,7 +4432,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>108</v>
       </c>
@@ -4261,7 +4455,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>112</v>
       </c>
@@ -4284,7 +4478,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>116</v>
       </c>
@@ -4307,7 +4501,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>120</v>
       </c>
@@ -4330,7 +4524,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>124</v>
       </c>
@@ -4353,7 +4547,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>128</v>
       </c>
@@ -4376,7 +4570,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>132</v>
       </c>
@@ -4399,7 +4593,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>136</v>
       </c>
@@ -4422,7 +4616,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
         <v>140</v>
       </c>
@@ -4445,7 +4639,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>144</v>
       </c>
@@ -4468,7 +4662,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
         <v>148</v>
       </c>
@@ -4491,7 +4685,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>150</v>
       </c>
@@ -4514,7 +4708,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
         <v>154</v>
       </c>
@@ -4537,7 +4731,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>158</v>
       </c>
@@ -4560,7 +4754,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
         <v>162</v>
       </c>
@@ -4583,7 +4777,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
         <v>166</v>
       </c>
@@ -4606,7 +4800,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>170</v>
       </c>
@@ -4629,7 +4823,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
         <v>172</v>
       </c>
@@ -4652,7 +4846,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
         <v>176</v>
       </c>
@@ -4675,7 +4869,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
         <v>180</v>
       </c>
@@ -4698,7 +4892,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
         <v>184</v>
       </c>
@@ -4721,7 +4915,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
         <v>188</v>
       </c>
@@ -4744,7 +4938,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
         <v>193</v>
       </c>
@@ -4767,7 +4961,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
         <v>197</v>
       </c>
@@ -4790,7 +4984,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
         <v>201</v>
       </c>
@@ -4813,7 +5007,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
         <v>205</v>
       </c>
@@ -4836,7 +5030,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
         <v>207</v>
       </c>
@@ -4859,7 +5053,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
         <v>211</v>
       </c>
@@ -4879,10 +5073,10 @@
         <v>215</v>
       </c>
       <c r="G57" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
         <v>216</v>
       </c>
@@ -4902,10 +5096,10 @@
         <v>215</v>
       </c>
       <c r="G58" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
         <v>218</v>
       </c>
@@ -4925,10 +5119,10 @@
         <v>215</v>
       </c>
       <c r="G59" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
         <v>220</v>
       </c>
@@ -4948,10 +5142,10 @@
         <v>215</v>
       </c>
       <c r="G60" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
         <v>222</v>
       </c>
@@ -4971,10 +5165,10 @@
         <v>215</v>
       </c>
       <c r="G61" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
         <v>224</v>
       </c>
@@ -4994,10 +5188,10 @@
         <v>215</v>
       </c>
       <c r="G62" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
         <v>226</v>
       </c>
@@ -5017,10 +5211,10 @@
         <v>215</v>
       </c>
       <c r="G63" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
         <v>228</v>
       </c>
@@ -5040,10 +5234,10 @@
         <v>215</v>
       </c>
       <c r="G64" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.35">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
         <v>230</v>
       </c>
@@ -5063,10 +5257,10 @@
         <v>215</v>
       </c>
       <c r="G65" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.35">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
         <v>232</v>
       </c>
@@ -5086,10 +5280,10 @@
         <v>215</v>
       </c>
       <c r="G66" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.35">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
         <v>234</v>
       </c>
@@ -5109,10 +5303,10 @@
         <v>215</v>
       </c>
       <c r="G67" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.35">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
         <v>236</v>
       </c>
@@ -5132,10 +5326,10 @@
         <v>215</v>
       </c>
       <c r="G68" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.35">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A69" s="1" t="s">
         <v>238</v>
       </c>
@@ -5155,10 +5349,10 @@
         <v>215</v>
       </c>
       <c r="G69" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.35">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A70" s="1" t="s">
         <v>240</v>
       </c>
@@ -5178,10 +5372,10 @@
         <v>215</v>
       </c>
       <c r="G70" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.35">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A71" s="1" t="s">
         <v>242</v>
       </c>
@@ -5201,10 +5395,10 @@
         <v>215</v>
       </c>
       <c r="G71" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.35">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A72" s="1" t="s">
         <v>244</v>
       </c>
@@ -5224,10 +5418,10 @@
         <v>215</v>
       </c>
       <c r="G72" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.35">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A73" s="1" t="s">
         <v>246</v>
       </c>
@@ -5247,10 +5441,10 @@
         <v>215</v>
       </c>
       <c r="G73" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.35">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A74" s="1" t="s">
         <v>248</v>
       </c>
@@ -5270,10 +5464,10 @@
         <v>215</v>
       </c>
       <c r="G74" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.35">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A75" s="1" t="s">
         <v>250</v>
       </c>
@@ -5293,10 +5487,10 @@
         <v>215</v>
       </c>
       <c r="G75" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.35">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A76" s="1" t="s">
         <v>252</v>
       </c>
@@ -5316,10 +5510,10 @@
         <v>215</v>
       </c>
       <c r="G76" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.35">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A77" s="1" t="s">
         <v>254</v>
       </c>
@@ -5339,10 +5533,10 @@
         <v>215</v>
       </c>
       <c r="G77" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.35">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A78" s="1" t="s">
         <v>256</v>
       </c>
@@ -5362,10 +5556,10 @@
         <v>215</v>
       </c>
       <c r="G78" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.35">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A79" s="1" t="s">
         <v>258</v>
       </c>
@@ -5385,10 +5579,10 @@
         <v>215</v>
       </c>
       <c r="G79" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.35">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A80" s="1" t="s">
         <v>260</v>
       </c>
@@ -5408,10 +5602,10 @@
         <v>215</v>
       </c>
       <c r="G80" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.35">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A81" s="1" t="s">
         <v>262</v>
       </c>
@@ -5431,10 +5625,10 @@
         <v>215</v>
       </c>
       <c r="G81" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.35">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A82" s="1" t="s">
         <v>264</v>
       </c>
@@ -5454,10 +5648,10 @@
         <v>215</v>
       </c>
       <c r="G82" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.35">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A83" s="1" t="s">
         <v>266</v>
       </c>
@@ -5477,10 +5671,10 @@
         <v>215</v>
       </c>
       <c r="G83" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.35">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A84" s="1" t="s">
         <v>268</v>
       </c>
@@ -5500,10 +5694,10 @@
         <v>215</v>
       </c>
       <c r="G84" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.35">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A85" s="1" t="s">
         <v>270</v>
       </c>
@@ -5523,10 +5717,10 @@
         <v>215</v>
       </c>
       <c r="G85" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.35">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A86" s="1" t="s">
         <v>272</v>
       </c>
@@ -5546,10 +5740,10 @@
         <v>215</v>
       </c>
       <c r="G86" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.35">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A87" s="1" t="s">
         <v>274</v>
       </c>
@@ -5569,10 +5763,10 @@
         <v>215</v>
       </c>
       <c r="G87" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.35">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A88" s="1" t="s">
         <v>276</v>
       </c>
@@ -5592,10 +5786,10 @@
         <v>215</v>
       </c>
       <c r="G88" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.35">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A89" s="1" t="s">
         <v>278</v>
       </c>
@@ -5615,10 +5809,10 @@
         <v>215</v>
       </c>
       <c r="G89" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.35">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A90" s="1" t="s">
         <v>280</v>
       </c>
@@ -5638,10 +5832,10 @@
         <v>215</v>
       </c>
       <c r="G90" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.35">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A91" s="1" t="s">
         <v>282</v>
       </c>
@@ -5664,7 +5858,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A92" s="1" t="s">
         <v>286</v>
       </c>
@@ -5687,7 +5881,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A93" s="1" t="s">
         <v>291</v>
       </c>
@@ -5710,7 +5904,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A94" s="1" t="s">
         <v>293</v>
       </c>
@@ -5733,7 +5927,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A95" s="1" t="s">
         <v>295</v>
       </c>
@@ -5756,7 +5950,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A96" s="1" t="s">
         <v>297</v>
       </c>
@@ -5779,7 +5973,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A97" s="1" t="s">
         <v>299</v>
       </c>
@@ -5802,7 +5996,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A98" s="1" t="s">
         <v>301</v>
       </c>
@@ -5825,7 +6019,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A99" s="1" t="s">
         <v>305</v>
       </c>
@@ -5848,7 +6042,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A100" s="1" t="s">
         <v>307</v>
       </c>
@@ -5871,7 +6065,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A101" s="1" t="s">
         <v>311</v>
       </c>
@@ -5894,7 +6088,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A102" s="1" t="s">
         <v>316</v>
       </c>
@@ -5917,7 +6111,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A103" s="1" t="s">
         <v>318</v>
       </c>
@@ -5940,7 +6134,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A104" s="1" t="s">
         <v>320</v>
       </c>
@@ -5963,7 +6157,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A105" s="1" t="s">
         <v>322</v>
       </c>
@@ -5986,7 +6180,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A106" s="1" t="s">
         <v>324</v>
       </c>
@@ -6009,7 +6203,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="107" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A107" s="1" t="s">
         <v>326</v>
       </c>
@@ -6032,7 +6226,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="108" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A108" s="1" t="s">
         <v>330</v>
       </c>
@@ -6055,7 +6249,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="109" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A109" s="1" t="s">
         <v>334</v>
       </c>
@@ -6078,7 +6272,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="110" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A110" s="1" t="s">
         <v>338</v>
       </c>
@@ -6101,7 +6295,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="111" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A111" s="1" t="s">
         <v>340</v>
       </c>
@@ -6124,7 +6318,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="112" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A112" s="1" t="s">
         <v>344</v>
       </c>
@@ -6147,7 +6341,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="113" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A113" s="1" t="s">
         <v>346</v>
       </c>
@@ -6170,7 +6364,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="114" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A114" s="1" t="s">
         <v>350</v>
       </c>
@@ -6193,7 +6387,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="115" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A115" s="1" t="s">
         <v>354</v>
       </c>
@@ -6216,7 +6410,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="116" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A116" s="1" t="s">
         <v>358</v>
       </c>
@@ -6239,7 +6433,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="117" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A117" s="1" t="s">
         <v>362</v>
       </c>
@@ -6262,7 +6456,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="118" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A118" s="1" t="s">
         <v>366</v>
       </c>
@@ -6285,7 +6479,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="119" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A119" s="1" t="s">
         <v>370</v>
       </c>
@@ -6308,7 +6502,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="120" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A120" s="1" t="s">
         <v>374</v>
       </c>
@@ -6331,7 +6525,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="121" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A121" s="1" t="s">
         <v>378</v>
       </c>
@@ -6354,7 +6548,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="122" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A122" s="1" t="s">
         <v>382</v>
       </c>
@@ -6377,7 +6571,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="123" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A123" s="1" t="s">
         <v>384</v>
       </c>
@@ -6400,7 +6594,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="124" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A124" s="1" t="s">
         <v>388</v>
       </c>
@@ -6423,7 +6617,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="125" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A125" s="1" t="s">
         <v>391</v>
       </c>
@@ -6446,7 +6640,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="126" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A126" s="1" t="s">
         <v>393</v>
       </c>
@@ -6469,7 +6663,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="127" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A127" s="1" t="s">
         <v>395</v>
       </c>
@@ -6492,7 +6686,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="128" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A128" s="1" t="s">
         <v>397</v>
       </c>
@@ -6515,7 +6709,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="129" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A129" s="1" t="s">
         <v>399</v>
       </c>
@@ -6538,7 +6732,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="130" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A130" s="1" t="s">
         <v>401</v>
       </c>
@@ -6561,7 +6755,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="131" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A131" s="1" t="s">
         <v>403</v>
       </c>
@@ -6584,7 +6778,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="132" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A132" s="1" t="s">
         <v>407</v>
       </c>
@@ -6607,7 +6801,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="133" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A133" s="1" t="s">
         <v>411</v>
       </c>
@@ -6630,7 +6824,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="134" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A134" s="1" t="s">
         <v>413</v>
       </c>
@@ -6653,7 +6847,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="135" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A135" s="1" t="s">
         <v>417</v>
       </c>
@@ -6676,7 +6870,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="136" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A136" s="1" t="s">
         <v>421</v>
       </c>
@@ -6699,7 +6893,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="137" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A137" s="1" t="s">
         <v>425</v>
       </c>
@@ -6722,7 +6916,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="138" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A138" s="1" t="s">
         <v>429</v>
       </c>
@@ -6745,7 +6939,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="139" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A139" s="1" t="s">
         <v>431</v>
       </c>
@@ -6768,7 +6962,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="140" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A140" s="1" t="s">
         <v>435</v>
       </c>
@@ -6791,7 +6985,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="141" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A141" s="1" t="s">
         <v>437</v>
       </c>
@@ -6814,7 +7008,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="142" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A142" s="1" t="s">
         <v>441</v>
       </c>
@@ -6837,7 +7031,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="143" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A143" s="1" t="s">
         <v>446</v>
       </c>
@@ -6860,7 +7054,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="144" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A144" s="1" t="s">
         <v>450</v>
       </c>
@@ -6883,7 +7077,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="145" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A145" s="1" t="s">
         <v>454</v>
       </c>
@@ -6906,7 +7100,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="146" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A146" s="1" t="s">
         <v>458</v>
       </c>
@@ -6929,7 +7123,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="147" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A147" s="1" t="s">
         <v>462</v>
       </c>
@@ -6952,7 +7146,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="148" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A148" s="1" t="s">
         <v>466</v>
       </c>
@@ -6975,7 +7169,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="149" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A149" s="1" t="s">
         <v>470</v>
       </c>
@@ -6998,7 +7192,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="150" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A150" s="1" t="s">
         <v>474</v>
       </c>
@@ -7021,7 +7215,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="151" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A151" s="1" t="s">
         <v>478</v>
       </c>
@@ -7044,7 +7238,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="152" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A152" s="1" t="s">
         <v>482</v>
       </c>
@@ -7067,7 +7261,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="153" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A153" s="1" t="s">
         <v>486</v>
       </c>
@@ -7090,7 +7284,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="154" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A154" s="1" t="s">
         <v>490</v>
       </c>
@@ -7113,7 +7307,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="155" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A155" s="1" t="s">
         <v>494</v>
       </c>
@@ -7136,7 +7330,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="156" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A156" s="1" t="s">
         <v>498</v>
       </c>
@@ -7159,7 +7353,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="157" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A157" s="1" t="s">
         <v>502</v>
       </c>
@@ -7182,7 +7376,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="158" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A158" s="1" t="s">
         <v>506</v>
       </c>
@@ -7205,7 +7399,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="159" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A159" s="1" t="s">
         <v>510</v>
       </c>
@@ -7228,7 +7422,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="160" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A160" s="1" t="s">
         <v>514</v>
       </c>
@@ -7251,7 +7445,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="161" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A161" s="1" t="s">
         <v>518</v>
       </c>
@@ -7274,7 +7468,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="162" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A162" s="1" t="s">
         <v>522</v>
       </c>
@@ -7297,7 +7491,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="163" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A163" s="1" t="s">
         <v>526</v>
       </c>
@@ -7320,7 +7514,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="164" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A164" s="1" t="s">
         <v>530</v>
       </c>
@@ -7343,7 +7537,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="165" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A165" s="1" t="s">
         <v>534</v>
       </c>
@@ -7366,7 +7560,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="166" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A166" s="1" t="s">
         <v>538</v>
       </c>
@@ -7389,7 +7583,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="167" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A167" s="1" t="s">
         <v>542</v>
       </c>
@@ -7412,7 +7606,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="168" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A168" s="1" t="s">
         <v>546</v>
       </c>
@@ -7435,7 +7629,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="169" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A169" s="1" t="s">
         <v>550</v>
       </c>
@@ -7458,7 +7652,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="170" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A170" s="1" t="s">
         <v>554</v>
       </c>
@@ -7481,7 +7675,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="171" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A171" s="1" t="s">
         <v>558</v>
       </c>
@@ -7504,7 +7698,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="172" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A172" s="1" t="s">
         <v>560</v>
       </c>
@@ -7527,7 +7721,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="173" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A173" s="1" t="s">
         <v>562</v>
       </c>
@@ -7550,7 +7744,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="174" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A174" s="1" t="s">
         <v>566</v>
       </c>
@@ -7573,7 +7767,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="175" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A175" s="1" t="s">
         <v>570</v>
       </c>
@@ -7596,7 +7790,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="176" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A176" s="1" t="s">
         <v>574</v>
       </c>
@@ -7619,7 +7813,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="177" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A177" s="1" t="s">
         <v>578</v>
       </c>
@@ -7642,7 +7836,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="178" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A178" s="1" t="s">
         <v>582</v>
       </c>
@@ -7665,7 +7859,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="179" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A179" s="1" t="s">
         <v>586</v>
       </c>
@@ -7688,7 +7882,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="180" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A180" s="1" t="s">
         <v>590</v>
       </c>
@@ -7711,7 +7905,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="181" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A181" s="1" t="s">
         <v>594</v>
       </c>
@@ -7734,7 +7928,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="182" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A182" s="1" t="s">
         <v>598</v>
       </c>
@@ -7757,7 +7951,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="183" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A183" s="1" t="s">
         <v>602</v>
       </c>
@@ -7780,7 +7974,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="184" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A184" s="1" t="s">
         <v>606</v>
       </c>
@@ -7794,16 +7988,16 @@
         <v>609</v>
       </c>
       <c r="E184" s="2" t="s">
-        <v>857</v>
+        <v>855</v>
       </c>
       <c r="F184" s="2" t="s">
-        <v>858</v>
+        <v>856</v>
       </c>
       <c r="G184" s="1" t="s">
-        <v>811</v>
-      </c>
-    </row>
-    <row r="185" spans="1:7" x14ac:dyDescent="0.35">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="185" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A185" s="1" t="s">
         <v>610</v>
       </c>
@@ -7817,16 +8011,16 @@
         <v>611</v>
       </c>
       <c r="E185" s="2" t="s">
-        <v>860</v>
+        <v>858</v>
       </c>
       <c r="F185" s="2" t="s">
-        <v>861</v>
+        <v>859</v>
       </c>
       <c r="G185" s="1" t="s">
-        <v>859</v>
-      </c>
-    </row>
-    <row r="186" spans="1:7" x14ac:dyDescent="0.35">
+        <v>857</v>
+      </c>
+    </row>
+    <row r="186" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A186" s="1" t="s">
         <v>612</v>
       </c>
@@ -7840,16 +8034,16 @@
         <v>613</v>
       </c>
       <c r="E186" s="2" t="s">
-        <v>857</v>
+        <v>855</v>
       </c>
       <c r="F186" s="2" t="s">
-        <v>862</v>
+        <v>860</v>
       </c>
       <c r="G186" s="1" t="s">
-        <v>811</v>
-      </c>
-    </row>
-    <row r="187" spans="1:7" x14ac:dyDescent="0.35">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="187" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A187" s="1" t="s">
         <v>614</v>
       </c>
@@ -7863,16 +8057,16 @@
         <v>615</v>
       </c>
       <c r="E187" s="2" t="s">
-        <v>857</v>
+        <v>855</v>
       </c>
       <c r="F187" s="2" t="s">
-        <v>863</v>
+        <v>861</v>
       </c>
       <c r="G187" s="1" t="s">
-        <v>811</v>
-      </c>
-    </row>
-    <row r="188" spans="1:7" x14ac:dyDescent="0.35">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="188" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A188" s="1" t="s">
         <v>616</v>
       </c>
@@ -7886,16 +8080,16 @@
         <v>617</v>
       </c>
       <c r="E188" s="2" t="s">
-        <v>864</v>
+        <v>862</v>
       </c>
       <c r="F188" s="2" t="s">
-        <v>865</v>
+        <v>863</v>
       </c>
       <c r="G188" s="1" t="s">
-        <v>811</v>
-      </c>
-    </row>
-    <row r="189" spans="1:7" x14ac:dyDescent="0.35">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="189" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A189" s="1" t="s">
         <v>618</v>
       </c>
@@ -7909,16 +8103,16 @@
         <v>619</v>
       </c>
       <c r="E189" s="2" t="s">
-        <v>867</v>
+        <v>865</v>
       </c>
       <c r="F189" s="2" t="s">
-        <v>868</v>
+        <v>866</v>
       </c>
       <c r="G189" s="1" t="s">
-        <v>866</v>
-      </c>
-    </row>
-    <row r="190" spans="1:7" x14ac:dyDescent="0.35">
+        <v>864</v>
+      </c>
+    </row>
+    <row r="190" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A190" s="1" t="s">
         <v>620</v>
       </c>
@@ -7932,16 +8126,16 @@
         <v>621</v>
       </c>
       <c r="E190" s="2" t="s">
-        <v>869</v>
+        <v>867</v>
       </c>
       <c r="F190" s="2" t="s">
-        <v>870</v>
+        <v>868</v>
       </c>
       <c r="G190" s="1" t="s">
-        <v>811</v>
-      </c>
-    </row>
-    <row r="191" spans="1:7" x14ac:dyDescent="0.35">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="191" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A191" s="1" t="s">
         <v>622</v>
       </c>
@@ -7955,16 +8149,16 @@
         <v>623</v>
       </c>
       <c r="E191" s="2" t="s">
-        <v>871</v>
+        <v>869</v>
       </c>
       <c r="F191" s="2" t="s">
-        <v>872</v>
+        <v>870</v>
       </c>
       <c r="G191" s="1" t="s">
-        <v>811</v>
-      </c>
-    </row>
-    <row r="192" spans="1:7" x14ac:dyDescent="0.35">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="192" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A192" s="1" t="s">
         <v>624</v>
       </c>
@@ -7978,16 +8172,16 @@
         <v>625</v>
       </c>
       <c r="E192" s="2" t="s">
-        <v>873</v>
+        <v>871</v>
       </c>
       <c r="F192" s="2" t="s">
-        <v>874</v>
+        <v>872</v>
       </c>
       <c r="G192" s="1" t="s">
-        <v>811</v>
-      </c>
-    </row>
-    <row r="193" spans="1:7" x14ac:dyDescent="0.35">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="193" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A193" s="1" t="s">
         <v>626</v>
       </c>
@@ -8010,7 +8204,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="194" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A194" s="1" t="s">
         <v>630</v>
       </c>
@@ -8033,7 +8227,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="195" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A195" s="1" t="s">
         <v>634</v>
       </c>
@@ -8056,7 +8250,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="196" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A196" s="1" t="s">
         <v>638</v>
       </c>
@@ -8079,7 +8273,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="197" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A197" s="1" t="s">
         <v>642</v>
       </c>
@@ -8102,7 +8296,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="198" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A198" s="1" t="s">
         <v>646</v>
       </c>
@@ -8125,7 +8319,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="199" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A199" s="1" t="s">
         <v>650</v>
       </c>
@@ -8148,7 +8342,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="200" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A200" s="1" t="s">
         <v>654</v>
       </c>
@@ -8171,7 +8365,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="201" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A201" s="1" t="s">
         <v>658</v>
       </c>
@@ -8194,7 +8388,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="202" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A202" s="1" t="s">
         <v>662</v>
       </c>
@@ -8217,7 +8411,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="203" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A203" s="1" t="s">
         <v>666</v>
       </c>
@@ -8240,7 +8434,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="204" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A204" s="1" t="s">
         <v>670</v>
       </c>
@@ -8254,18 +8448,18 @@
         <v>672</v>
       </c>
       <c r="E204" s="2" t="s">
+        <v>873</v>
+      </c>
+      <c r="F204" s="2" t="s">
+        <v>874</v>
+      </c>
+      <c r="G204" s="1" t="s">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="205" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A205" s="1" t="s">
         <v>673</v>
-      </c>
-      <c r="F204" s="2" t="s">
-        <v>674</v>
-      </c>
-      <c r="G204" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="205" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A205" s="1" t="s">
-        <v>675</v>
       </c>
       <c r="B205" s="1" t="s">
         <v>607</v>
@@ -8274,21 +8468,21 @@
         <v>671</v>
       </c>
       <c r="D205" s="1" t="s">
-        <v>676</v>
+        <v>674</v>
       </c>
       <c r="E205" s="2" t="s">
-        <v>673</v>
+        <v>875</v>
       </c>
       <c r="F205" s="2" t="s">
-        <v>674</v>
+        <v>876</v>
       </c>
       <c r="G205" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="206" spans="1:7" x14ac:dyDescent="0.35">
+        <v>877</v>
+      </c>
+    </row>
+    <row r="206" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A206" s="1" t="s">
-        <v>677</v>
+        <v>675</v>
       </c>
       <c r="B206" s="1" t="s">
         <v>607</v>
@@ -8297,21 +8491,21 @@
         <v>671</v>
       </c>
       <c r="D206" s="1" t="s">
-        <v>678</v>
+        <v>676</v>
       </c>
       <c r="E206" s="2" t="s">
-        <v>673</v>
+        <v>878</v>
       </c>
       <c r="F206" s="2" t="s">
-        <v>674</v>
+        <v>879</v>
       </c>
       <c r="G206" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="207" spans="1:7" x14ac:dyDescent="0.35">
+        <v>880</v>
+      </c>
+    </row>
+    <row r="207" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A207" s="1" t="s">
-        <v>679</v>
+        <v>677</v>
       </c>
       <c r="B207" s="1" t="s">
         <v>607</v>
@@ -8320,21 +8514,21 @@
         <v>671</v>
       </c>
       <c r="D207" s="1" t="s">
-        <v>680</v>
+        <v>678</v>
       </c>
       <c r="E207" s="2" t="s">
-        <v>673</v>
+        <v>881</v>
       </c>
       <c r="F207" s="2" t="s">
-        <v>674</v>
+        <v>882</v>
       </c>
       <c r="G207" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="208" spans="1:7" x14ac:dyDescent="0.35">
+        <v>883</v>
+      </c>
+    </row>
+    <row r="208" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A208" s="1" t="s">
-        <v>681</v>
+        <v>679</v>
       </c>
       <c r="B208" s="1" t="s">
         <v>607</v>
@@ -8343,21 +8537,21 @@
         <v>671</v>
       </c>
       <c r="D208" s="1" t="s">
-        <v>682</v>
+        <v>680</v>
       </c>
       <c r="E208" s="2" t="s">
-        <v>673</v>
+        <v>884</v>
       </c>
       <c r="F208" s="2" t="s">
-        <v>674</v>
+        <v>885</v>
       </c>
       <c r="G208" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="209" spans="1:7" x14ac:dyDescent="0.35">
+        <v>886</v>
+      </c>
+    </row>
+    <row r="209" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A209" s="1" t="s">
-        <v>683</v>
+        <v>681</v>
       </c>
       <c r="B209" s="1" t="s">
         <v>607</v>
@@ -8366,21 +8560,21 @@
         <v>671</v>
       </c>
       <c r="D209" s="1" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="E209" s="2" t="s">
-        <v>673</v>
+        <v>887</v>
       </c>
       <c r="F209" s="2" t="s">
-        <v>674</v>
+        <v>888</v>
       </c>
       <c r="G209" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="210" spans="1:7" x14ac:dyDescent="0.35">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="210" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A210" s="1" t="s">
-        <v>685</v>
+        <v>683</v>
       </c>
       <c r="B210" s="1" t="s">
         <v>607</v>
@@ -8389,21 +8583,21 @@
         <v>671</v>
       </c>
       <c r="D210" s="1" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
       <c r="E210" s="2" t="s">
-        <v>673</v>
+        <v>889</v>
       </c>
       <c r="F210" s="2" t="s">
-        <v>674</v>
+        <v>890</v>
       </c>
       <c r="G210" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="211" spans="1:7" x14ac:dyDescent="0.35">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="211" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A211" s="1" t="s">
-        <v>687</v>
+        <v>685</v>
       </c>
       <c r="B211" s="1" t="s">
         <v>607</v>
@@ -8412,21 +8606,21 @@
         <v>671</v>
       </c>
       <c r="D211" s="1" t="s">
-        <v>688</v>
+        <v>686</v>
       </c>
       <c r="E211" s="2" t="s">
-        <v>673</v>
+        <v>891</v>
       </c>
       <c r="F211" s="2" t="s">
-        <v>674</v>
+        <v>892</v>
       </c>
       <c r="G211" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="212" spans="1:7" x14ac:dyDescent="0.35">
+        <v>893</v>
+      </c>
+    </row>
+    <row r="212" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A212" s="1" t="s">
-        <v>689</v>
+        <v>687</v>
       </c>
       <c r="B212" s="1" t="s">
         <v>607</v>
@@ -8435,21 +8629,21 @@
         <v>671</v>
       </c>
       <c r="D212" s="1" t="s">
-        <v>690</v>
+        <v>688</v>
       </c>
       <c r="E212" s="2" t="s">
-        <v>673</v>
+        <v>894</v>
       </c>
       <c r="F212" s="2" t="s">
-        <v>674</v>
+        <v>895</v>
       </c>
       <c r="G212" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="213" spans="1:7" x14ac:dyDescent="0.35">
+        <v>896</v>
+      </c>
+    </row>
+    <row r="213" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A213" s="1" t="s">
-        <v>691</v>
+        <v>689</v>
       </c>
       <c r="B213" s="1" t="s">
         <v>607</v>
@@ -8458,21 +8652,21 @@
         <v>671</v>
       </c>
       <c r="D213" s="1" t="s">
-        <v>692</v>
+        <v>690</v>
       </c>
       <c r="E213" s="2" t="s">
-        <v>673</v>
+        <v>897</v>
       </c>
       <c r="F213" s="2" t="s">
-        <v>674</v>
+        <v>898</v>
       </c>
       <c r="G213" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="214" spans="1:7" x14ac:dyDescent="0.35">
+        <v>899</v>
+      </c>
+    </row>
+    <row r="214" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A214" s="1" t="s">
-        <v>693</v>
+        <v>691</v>
       </c>
       <c r="B214" s="1" t="s">
         <v>607</v>
@@ -8481,21 +8675,21 @@
         <v>671</v>
       </c>
       <c r="D214" s="1" t="s">
-        <v>694</v>
+        <v>692</v>
       </c>
       <c r="E214" s="2" t="s">
-        <v>673</v>
+        <v>900</v>
       </c>
       <c r="F214" s="2" t="s">
-        <v>674</v>
+        <v>901</v>
       </c>
       <c r="G214" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="215" spans="1:7" x14ac:dyDescent="0.35">
+        <v>902</v>
+      </c>
+    </row>
+    <row r="215" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A215" s="1" t="s">
-        <v>695</v>
+        <v>693</v>
       </c>
       <c r="B215" s="1" t="s">
         <v>607</v>
@@ -8504,21 +8698,21 @@
         <v>671</v>
       </c>
       <c r="D215" s="1" t="s">
-        <v>696</v>
+        <v>694</v>
       </c>
       <c r="E215" s="2" t="s">
-        <v>673</v>
+        <v>903</v>
       </c>
       <c r="F215" s="2" t="s">
-        <v>674</v>
+        <v>904</v>
       </c>
       <c r="G215" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="216" spans="1:7" x14ac:dyDescent="0.35">
+        <v>905</v>
+      </c>
+    </row>
+    <row r="216" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A216" s="1" t="s">
-        <v>697</v>
+        <v>695</v>
       </c>
       <c r="B216" s="1" t="s">
         <v>607</v>
@@ -8527,21 +8721,21 @@
         <v>671</v>
       </c>
       <c r="D216" s="1" t="s">
-        <v>698</v>
+        <v>696</v>
       </c>
       <c r="E216" s="2" t="s">
-        <v>673</v>
+        <v>906</v>
       </c>
       <c r="F216" s="2" t="s">
-        <v>674</v>
+        <v>907</v>
       </c>
       <c r="G216" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="217" spans="1:7" x14ac:dyDescent="0.35">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="217" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A217" s="1" t="s">
-        <v>699</v>
+        <v>697</v>
       </c>
       <c r="B217" s="1" t="s">
         <v>607</v>
@@ -8550,21 +8744,21 @@
         <v>671</v>
       </c>
       <c r="D217" s="1" t="s">
-        <v>700</v>
+        <v>698</v>
       </c>
       <c r="E217" s="2" t="s">
-        <v>673</v>
+        <v>908</v>
       </c>
       <c r="F217" s="2" t="s">
-        <v>674</v>
+        <v>909</v>
       </c>
       <c r="G217" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="218" spans="1:7" x14ac:dyDescent="0.35">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="218" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A218" s="1" t="s">
-        <v>701</v>
+        <v>699</v>
       </c>
       <c r="B218" s="1" t="s">
         <v>607</v>
@@ -8573,21 +8767,21 @@
         <v>671</v>
       </c>
       <c r="D218" s="1" t="s">
-        <v>702</v>
+        <v>700</v>
       </c>
       <c r="E218" s="2" t="s">
-        <v>673</v>
+        <v>911</v>
       </c>
       <c r="F218" s="2" t="s">
-        <v>674</v>
+        <v>912</v>
       </c>
       <c r="G218" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="219" spans="1:7" x14ac:dyDescent="0.35">
+        <v>913</v>
+      </c>
+    </row>
+    <row r="219" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A219" s="1" t="s">
-        <v>703</v>
+        <v>701</v>
       </c>
       <c r="B219" s="1" t="s">
         <v>607</v>
@@ -8596,21 +8790,21 @@
         <v>671</v>
       </c>
       <c r="D219" s="1" t="s">
-        <v>704</v>
+        <v>702</v>
       </c>
       <c r="E219" s="2" t="s">
-        <v>673</v>
+        <v>914</v>
       </c>
       <c r="F219" s="2" t="s">
-        <v>674</v>
+        <v>915</v>
       </c>
       <c r="G219" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="220" spans="1:7" x14ac:dyDescent="0.35">
+        <v>916</v>
+      </c>
+    </row>
+    <row r="220" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A220" s="1" t="s">
-        <v>705</v>
+        <v>703</v>
       </c>
       <c r="B220" s="1" t="s">
         <v>607</v>
@@ -8619,21 +8813,21 @@
         <v>671</v>
       </c>
       <c r="D220" s="1" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="E220" s="2" t="s">
-        <v>673</v>
+        <v>917</v>
       </c>
       <c r="F220" s="2" t="s">
-        <v>674</v>
+        <v>918</v>
       </c>
       <c r="G220" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="221" spans="1:7" x14ac:dyDescent="0.35">
+        <v>919</v>
+      </c>
+    </row>
+    <row r="221" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A221" s="1" t="s">
-        <v>707</v>
+        <v>705</v>
       </c>
       <c r="B221" s="1" t="s">
         <v>607</v>
@@ -8642,21 +8836,21 @@
         <v>671</v>
       </c>
       <c r="D221" s="1" t="s">
-        <v>708</v>
+        <v>706</v>
       </c>
       <c r="E221" s="2" t="s">
-        <v>673</v>
+        <v>920</v>
       </c>
       <c r="F221" s="2" t="s">
-        <v>674</v>
+        <v>921</v>
       </c>
       <c r="G221" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="222" spans="1:7" x14ac:dyDescent="0.35">
+        <v>922</v>
+      </c>
+    </row>
+    <row r="222" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A222" s="1" t="s">
-        <v>709</v>
+        <v>707</v>
       </c>
       <c r="B222" s="1" t="s">
         <v>607</v>
@@ -8665,21 +8859,21 @@
         <v>671</v>
       </c>
       <c r="D222" s="1" t="s">
-        <v>710</v>
+        <v>708</v>
       </c>
       <c r="E222" s="2" t="s">
-        <v>673</v>
+        <v>923</v>
       </c>
       <c r="F222" s="2" t="s">
-        <v>674</v>
+        <v>924</v>
       </c>
       <c r="G222" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="223" spans="1:7" x14ac:dyDescent="0.35">
+        <v>925</v>
+      </c>
+    </row>
+    <row r="223" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A223" s="1" t="s">
-        <v>711</v>
+        <v>709</v>
       </c>
       <c r="B223" s="1" t="s">
         <v>607</v>
@@ -8688,21 +8882,21 @@
         <v>671</v>
       </c>
       <c r="D223" s="1" t="s">
-        <v>712</v>
+        <v>710</v>
       </c>
       <c r="E223" s="2" t="s">
-        <v>673</v>
+        <v>926</v>
       </c>
       <c r="F223" s="2" t="s">
-        <v>674</v>
+        <v>927</v>
       </c>
       <c r="G223" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="224" spans="1:7" x14ac:dyDescent="0.35">
+        <v>928</v>
+      </c>
+    </row>
+    <row r="224" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A224" s="1" t="s">
-        <v>713</v>
+        <v>711</v>
       </c>
       <c r="B224" s="1" t="s">
         <v>607</v>
@@ -8711,21 +8905,21 @@
         <v>671</v>
       </c>
       <c r="D224" s="1" t="s">
-        <v>714</v>
+        <v>712</v>
       </c>
       <c r="E224" s="2" t="s">
-        <v>673</v>
+        <v>929</v>
       </c>
       <c r="F224" s="2" t="s">
-        <v>674</v>
+        <v>930</v>
       </c>
       <c r="G224" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="225" spans="1:7" x14ac:dyDescent="0.35">
+        <v>931</v>
+      </c>
+    </row>
+    <row r="225" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A225" s="1" t="s">
-        <v>715</v>
+        <v>713</v>
       </c>
       <c r="B225" s="1" t="s">
         <v>607</v>
@@ -8734,21 +8928,21 @@
         <v>671</v>
       </c>
       <c r="D225" s="1" t="s">
-        <v>716</v>
+        <v>714</v>
       </c>
       <c r="E225" s="2" t="s">
-        <v>673</v>
+        <v>932</v>
       </c>
       <c r="F225" s="2" t="s">
-        <v>674</v>
+        <v>933</v>
       </c>
       <c r="G225" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="226" spans="1:7" x14ac:dyDescent="0.35">
+        <v>934</v>
+      </c>
+    </row>
+    <row r="226" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A226" s="1" t="s">
-        <v>717</v>
+        <v>715</v>
       </c>
       <c r="B226" s="1" t="s">
         <v>607</v>
@@ -8757,21 +8951,21 @@
         <v>671</v>
       </c>
       <c r="D226" s="1" t="s">
-        <v>718</v>
+        <v>716</v>
       </c>
       <c r="E226" s="2" t="s">
-        <v>673</v>
+        <v>935</v>
       </c>
       <c r="F226" s="2" t="s">
-        <v>674</v>
+        <v>936</v>
       </c>
       <c r="G226" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="227" spans="1:7" x14ac:dyDescent="0.35">
+        <v>937</v>
+      </c>
+    </row>
+    <row r="227" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A227" s="1" t="s">
-        <v>719</v>
+        <v>717</v>
       </c>
       <c r="B227" s="1" t="s">
         <v>607</v>
@@ -8780,30 +8974,30 @@
         <v>671</v>
       </c>
       <c r="D227" s="1" t="s">
+        <v>718</v>
+      </c>
+      <c r="E227" s="2" t="s">
+        <v>938</v>
+      </c>
+      <c r="F227" s="2" t="s">
+        <v>939</v>
+      </c>
+      <c r="G227" s="1" t="s">
+        <v>940</v>
+      </c>
+    </row>
+    <row r="228" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A228" s="1" t="s">
+        <v>719</v>
+      </c>
+      <c r="B228" s="1" t="s">
         <v>720</v>
       </c>
-      <c r="E227" s="2" t="s">
-        <v>673</v>
-      </c>
-      <c r="F227" s="2" t="s">
-        <v>674</v>
-      </c>
-      <c r="G227" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="228" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A228" s="1" t="s">
+      <c r="C228" s="1" t="s">
         <v>721</v>
       </c>
-      <c r="B228" s="1" t="s">
-        <v>722</v>
-      </c>
-      <c r="C228" s="1" t="s">
-        <v>723</v>
-      </c>
       <c r="D228" s="1" t="s">
-        <v>723</v>
+        <v>721</v>
       </c>
       <c r="E228" s="2">
         <v>-79.406307499999997</v>
@@ -8812,596 +9006,596 @@
         <v>0.31493120000000002</v>
       </c>
       <c r="G228" s="1" t="s">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="229" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A229" s="1" t="s">
+        <v>722</v>
+      </c>
+      <c r="B229" s="1" t="s">
+        <v>720</v>
+      </c>
+      <c r="C229" s="1" t="s">
+        <v>723</v>
+      </c>
+      <c r="D229" s="1" t="s">
+        <v>724</v>
+      </c>
+      <c r="E229" s="2" t="s">
         <v>811</v>
       </c>
-    </row>
-    <row r="229" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A229" s="1" t="s">
-        <v>724</v>
-      </c>
-      <c r="B229" s="1" t="s">
-        <v>722</v>
-      </c>
-      <c r="C229" s="1" t="s">
+      <c r="F229" s="2" t="s">
+        <v>812</v>
+      </c>
+      <c r="G229" s="1" t="s">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="230" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A230" s="1" t="s">
         <v>725</v>
       </c>
-      <c r="D229" s="1" t="s">
+      <c r="B230" s="1" t="s">
+        <v>720</v>
+      </c>
+      <c r="C230" s="1" t="s">
+        <v>723</v>
+      </c>
+      <c r="D230" s="1" t="s">
         <v>726</v>
       </c>
-      <c r="E229" s="2" t="s">
+      <c r="E230" s="2" t="s">
         <v>813</v>
       </c>
-      <c r="F229" s="2" t="s">
+      <c r="F230" s="2" t="s">
         <v>814</v>
       </c>
-      <c r="G229" s="1" t="s">
-        <v>811</v>
-      </c>
-    </row>
-    <row r="230" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A230" s="1" t="s">
+      <c r="G230" s="1" t="s">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="231" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A231" s="1" t="s">
         <v>727</v>
       </c>
-      <c r="B230" s="1" t="s">
-        <v>722</v>
-      </c>
-      <c r="C230" s="1" t="s">
-        <v>725</v>
-      </c>
-      <c r="D230" s="1" t="s">
+      <c r="B231" s="1" t="s">
+        <v>720</v>
+      </c>
+      <c r="C231" s="1" t="s">
+        <v>723</v>
+      </c>
+      <c r="D231" s="1" t="s">
         <v>728</v>
       </c>
-      <c r="E230" s="2" t="s">
+      <c r="E231" s="2" t="s">
         <v>815</v>
       </c>
-      <c r="F230" s="2" t="s">
+      <c r="F231" s="2" t="s">
         <v>816</v>
       </c>
-      <c r="G230" s="1" t="s">
-        <v>811</v>
-      </c>
-    </row>
-    <row r="231" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A231" s="1" t="s">
+      <c r="G231" s="1" t="s">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="232" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A232" s="1" t="s">
         <v>729</v>
       </c>
-      <c r="B231" s="1" t="s">
-        <v>722</v>
-      </c>
-      <c r="C231" s="1" t="s">
-        <v>725</v>
-      </c>
-      <c r="D231" s="1" t="s">
+      <c r="B232" s="1" t="s">
+        <v>720</v>
+      </c>
+      <c r="C232" s="1" t="s">
+        <v>723</v>
+      </c>
+      <c r="D232" s="1" t="s">
         <v>730</v>
       </c>
-      <c r="E231" s="2" t="s">
+      <c r="E232" s="2" t="s">
         <v>817</v>
       </c>
-      <c r="F231" s="2" t="s">
+      <c r="F232" s="2" t="s">
         <v>818</v>
       </c>
-      <c r="G231" s="1" t="s">
-        <v>811</v>
-      </c>
-    </row>
-    <row r="232" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A232" s="1" t="s">
+      <c r="G232" s="1" t="s">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="233" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A233" s="1" t="s">
         <v>731</v>
       </c>
-      <c r="B232" s="1" t="s">
-        <v>722</v>
-      </c>
-      <c r="C232" s="1" t="s">
-        <v>725</v>
-      </c>
-      <c r="D232" s="1" t="s">
+      <c r="B233" s="1" t="s">
+        <v>720</v>
+      </c>
+      <c r="C233" s="1" t="s">
+        <v>723</v>
+      </c>
+      <c r="D233" s="1" t="s">
         <v>732</v>
       </c>
-      <c r="E232" s="2" t="s">
+      <c r="E233" s="2" t="s">
         <v>819</v>
       </c>
-      <c r="F232" s="2" t="s">
+      <c r="F233" s="2" t="s">
         <v>820</v>
       </c>
-      <c r="G232" s="1" t="s">
-        <v>811</v>
-      </c>
-    </row>
-    <row r="233" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A233" s="1" t="s">
+      <c r="G233" s="1" t="s">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="234" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A234" s="1" t="s">
         <v>733</v>
       </c>
-      <c r="B233" s="1" t="s">
-        <v>722</v>
-      </c>
-      <c r="C233" s="1" t="s">
-        <v>725</v>
-      </c>
-      <c r="D233" s="1" t="s">
+      <c r="B234" s="1" t="s">
+        <v>720</v>
+      </c>
+      <c r="C234" s="1" t="s">
+        <v>723</v>
+      </c>
+      <c r="D234" s="1" t="s">
         <v>734</v>
       </c>
-      <c r="E233" s="2" t="s">
+      <c r="E234" s="2" t="s">
         <v>821</v>
       </c>
-      <c r="F233" s="2" t="s">
+      <c r="F234" s="2" t="s">
         <v>822</v>
       </c>
-      <c r="G233" s="1" t="s">
-        <v>811</v>
-      </c>
-    </row>
-    <row r="234" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A234" s="1" t="s">
+      <c r="G234" s="1" t="s">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="235" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A235" s="1" t="s">
         <v>735</v>
       </c>
-      <c r="B234" s="1" t="s">
-        <v>722</v>
-      </c>
-      <c r="C234" s="1" t="s">
-        <v>725</v>
-      </c>
-      <c r="D234" s="1" t="s">
+      <c r="B235" s="1" t="s">
+        <v>720</v>
+      </c>
+      <c r="C235" s="1" t="s">
+        <v>723</v>
+      </c>
+      <c r="D235" s="1" t="s">
         <v>736</v>
       </c>
-      <c r="E234" s="2" t="s">
+      <c r="E235" s="2" t="s">
         <v>823</v>
       </c>
-      <c r="F234" s="2" t="s">
+      <c r="F235" s="2" t="s">
         <v>824</v>
       </c>
-      <c r="G234" s="1" t="s">
-        <v>811</v>
-      </c>
-    </row>
-    <row r="235" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A235" s="1" t="s">
+      <c r="G235" s="1" t="s">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="236" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A236" s="1" t="s">
         <v>737</v>
       </c>
-      <c r="B235" s="1" t="s">
-        <v>722</v>
-      </c>
-      <c r="C235" s="1" t="s">
-        <v>725</v>
-      </c>
-      <c r="D235" s="1" t="s">
+      <c r="B236" s="1" t="s">
+        <v>720</v>
+      </c>
+      <c r="C236" s="1" t="s">
         <v>738</v>
       </c>
-      <c r="E235" s="2" t="s">
-        <v>825</v>
-      </c>
-      <c r="F235" s="2" t="s">
-        <v>826</v>
-      </c>
-      <c r="G235" s="1" t="s">
-        <v>811</v>
-      </c>
-    </row>
-    <row r="236" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A236" s="1" t="s">
+      <c r="D236" s="1" t="s">
+        <v>738</v>
+      </c>
+      <c r="E236" s="2" t="s">
         <v>739</v>
       </c>
-      <c r="B236" s="1" t="s">
-        <v>722</v>
-      </c>
-      <c r="C236" s="1" t="s">
+      <c r="F236" s="2" t="s">
         <v>740</v>
       </c>
-      <c r="D236" s="1" t="s">
-        <v>740</v>
-      </c>
-      <c r="E236" s="2" t="s">
+      <c r="G236" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="237" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A237" s="1" t="s">
         <v>741</v>
       </c>
-      <c r="F236" s="2" t="s">
+      <c r="B237" s="1" t="s">
+        <v>720</v>
+      </c>
+      <c r="C237" s="1" t="s">
         <v>742</v>
       </c>
-      <c r="G236" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="237" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A237" s="1" t="s">
+      <c r="D237" s="1" t="s">
+        <v>742</v>
+      </c>
+      <c r="E237" s="2" t="s">
         <v>743</v>
       </c>
-      <c r="B237" s="1" t="s">
-        <v>722</v>
-      </c>
-      <c r="C237" s="1" t="s">
+      <c r="F237" s="2" t="s">
         <v>744</v>
       </c>
-      <c r="D237" s="1" t="s">
-        <v>744</v>
-      </c>
-      <c r="E237" s="2" t="s">
+      <c r="G237" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="238" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A238" s="1" t="s">
         <v>745</v>
       </c>
-      <c r="F237" s="2" t="s">
+      <c r="B238" s="1" t="s">
+        <v>720</v>
+      </c>
+      <c r="C238" s="1" t="s">
         <v>746</v>
       </c>
-      <c r="G237" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="238" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A238" s="1" t="s">
+      <c r="D238" s="1" t="s">
+        <v>746</v>
+      </c>
+      <c r="E238" s="2" t="s">
         <v>747</v>
       </c>
-      <c r="B238" s="1" t="s">
-        <v>722</v>
-      </c>
-      <c r="C238" s="1" t="s">
+      <c r="F238" s="2" t="s">
         <v>748</v>
       </c>
-      <c r="D238" s="1" t="s">
-        <v>748</v>
-      </c>
-      <c r="E238" s="2" t="s">
+      <c r="G238" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="239" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A239" s="1" t="s">
         <v>749</v>
       </c>
-      <c r="F238" s="2" t="s">
+      <c r="B239" s="1" t="s">
         <v>750</v>
       </c>
-      <c r="G238" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="239" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A239" s="1" t="s">
+      <c r="C239" s="1" t="s">
         <v>751</v>
       </c>
-      <c r="B239" s="1" t="s">
+      <c r="D239" s="1" t="s">
+        <v>751</v>
+      </c>
+      <c r="E239" s="2" t="s">
         <v>752</v>
       </c>
-      <c r="C239" s="1" t="s">
+      <c r="F239" s="2" t="s">
         <v>753</v>
       </c>
-      <c r="D239" s="1" t="s">
-        <v>753</v>
-      </c>
-      <c r="E239" s="2" t="s">
+      <c r="G239" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="240" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A240" s="1" t="s">
         <v>754</v>
       </c>
-      <c r="F239" s="2" t="s">
+      <c r="B240" s="1" t="s">
+        <v>750</v>
+      </c>
+      <c r="C240" s="1" t="s">
         <v>755</v>
       </c>
-      <c r="G239" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="240" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A240" s="1" t="s">
+      <c r="D240" s="1" t="s">
+        <v>755</v>
+      </c>
+      <c r="E240" s="2" t="s">
         <v>756</v>
       </c>
-      <c r="B240" s="1" t="s">
-        <v>752</v>
-      </c>
-      <c r="C240" s="1" t="s">
+      <c r="F240" s="2" t="s">
         <v>757</v>
       </c>
-      <c r="D240" s="1" t="s">
-        <v>757</v>
-      </c>
-      <c r="E240" s="2" t="s">
+      <c r="G240" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="241" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A241" s="1" t="s">
         <v>758</v>
       </c>
-      <c r="F240" s="2" t="s">
+      <c r="B241" s="1" t="s">
+        <v>750</v>
+      </c>
+      <c r="C241" s="1" t="s">
         <v>759</v>
       </c>
-      <c r="G240" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="241" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A241" s="1" t="s">
+      <c r="D241" s="1" t="s">
         <v>760</v>
       </c>
-      <c r="B241" s="1" t="s">
-        <v>752</v>
-      </c>
-      <c r="C241" s="1" t="s">
+      <c r="E241" s="2" t="s">
+        <v>828</v>
+      </c>
+      <c r="F241" s="2" t="s">
+        <v>829</v>
+      </c>
+      <c r="G241" s="1" t="s">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="242" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A242" s="1" t="s">
         <v>761</v>
       </c>
-      <c r="D241" s="1" t="s">
+      <c r="B242" s="1" t="s">
+        <v>750</v>
+      </c>
+      <c r="C242" s="1" t="s">
+        <v>759</v>
+      </c>
+      <c r="D242" s="1" t="s">
         <v>762</v>
       </c>
-      <c r="E241" s="2" t="s">
-        <v>830</v>
-      </c>
-      <c r="F241" s="2" t="s">
+      <c r="E242" s="2" t="s">
         <v>831</v>
       </c>
-      <c r="G241" s="1" t="s">
+      <c r="F242" s="2" t="s">
         <v>832</v>
       </c>
-    </row>
-    <row r="242" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A242" s="1" t="s">
+      <c r="G242" s="1" t="s">
+        <v>833</v>
+      </c>
+    </row>
+    <row r="243" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A243" s="1" t="s">
         <v>763</v>
       </c>
-      <c r="B242" s="1" t="s">
-        <v>752</v>
-      </c>
-      <c r="C242" s="1" t="s">
-        <v>761</v>
-      </c>
-      <c r="D242" s="1" t="s">
+      <c r="B243" s="1" t="s">
+        <v>750</v>
+      </c>
+      <c r="C243" s="1" t="s">
+        <v>759</v>
+      </c>
+      <c r="D243" s="1" t="s">
         <v>764</v>
       </c>
-      <c r="E242" s="2" t="s">
-        <v>833</v>
-      </c>
-      <c r="F242" s="2" t="s">
+      <c r="E243" s="2" t="s">
+        <v>837</v>
+      </c>
+      <c r="F243" s="2" t="s">
+        <v>838</v>
+      </c>
+      <c r="G243" s="1" t="s">
         <v>834</v>
       </c>
-      <c r="G242" s="1" t="s">
+    </row>
+    <row r="244" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A244" s="1" t="s">
+        <v>765</v>
+      </c>
+      <c r="B244" s="1" t="s">
+        <v>750</v>
+      </c>
+      <c r="C244" s="1" t="s">
+        <v>759</v>
+      </c>
+      <c r="D244" s="1" t="s">
+        <v>766</v>
+      </c>
+      <c r="E244" s="2" t="s">
+        <v>839</v>
+      </c>
+      <c r="F244" s="2" t="s">
+        <v>840</v>
+      </c>
+      <c r="G244" s="1" t="s">
         <v>835</v>
       </c>
     </row>
-    <row r="243" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A243" s="1" t="s">
-        <v>765</v>
-      </c>
-      <c r="B243" s="1" t="s">
-        <v>752</v>
-      </c>
-      <c r="C243" s="1" t="s">
-        <v>761</v>
-      </c>
-      <c r="D243" s="1" t="s">
-        <v>766</v>
-      </c>
-      <c r="E243" s="2" t="s">
-        <v>839</v>
-      </c>
-      <c r="F243" s="2" t="s">
-        <v>840</v>
-      </c>
-      <c r="G243" s="1" t="s">
+    <row r="245" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A245" s="1" t="s">
+        <v>767</v>
+      </c>
+      <c r="B245" s="1" t="s">
+        <v>750</v>
+      </c>
+      <c r="C245" s="1" t="s">
+        <v>759</v>
+      </c>
+      <c r="D245" s="1" t="s">
+        <v>768</v>
+      </c>
+      <c r="E245" s="2" t="s">
+        <v>841</v>
+      </c>
+      <c r="F245" s="2" t="s">
+        <v>842</v>
+      </c>
+      <c r="G245" s="1" t="s">
         <v>836</v>
       </c>
     </row>
-    <row r="244" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A244" s="1" t="s">
-        <v>767</v>
-      </c>
-      <c r="B244" s="1" t="s">
-        <v>752</v>
-      </c>
-      <c r="C244" s="1" t="s">
-        <v>761</v>
-      </c>
-      <c r="D244" s="1" t="s">
-        <v>768</v>
-      </c>
-      <c r="E244" s="2" t="s">
-        <v>841</v>
-      </c>
-      <c r="F244" s="2" t="s">
-        <v>842</v>
-      </c>
-      <c r="G244" s="1" t="s">
-        <v>837</v>
-      </c>
-    </row>
-    <row r="245" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A245" s="1" t="s">
+    <row r="246" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A246" s="1" t="s">
         <v>769</v>
       </c>
-      <c r="B245" s="1" t="s">
-        <v>752</v>
-      </c>
-      <c r="C245" s="1" t="s">
-        <v>761</v>
-      </c>
-      <c r="D245" s="1" t="s">
-        <v>770</v>
-      </c>
-      <c r="E245" s="2" t="s">
-        <v>843</v>
-      </c>
-      <c r="F245" s="2" t="s">
-        <v>844</v>
-      </c>
-      <c r="G245" s="1" t="s">
-        <v>838</v>
-      </c>
-    </row>
-    <row r="246" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A246" s="1" t="s">
-        <v>771</v>
-      </c>
       <c r="B246" s="1" t="s">
-        <v>752</v>
+        <v>750</v>
       </c>
       <c r="C246" s="1" t="s">
-        <v>761</v>
+        <v>759</v>
       </c>
       <c r="D246" s="1" t="s">
         <v>292</v>
       </c>
       <c r="E246" s="2" t="s">
+        <v>844</v>
+      </c>
+      <c r="F246" s="2" t="s">
+        <v>845</v>
+      </c>
+      <c r="G246" s="1" t="s">
+        <v>843</v>
+      </c>
+    </row>
+    <row r="247" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A247" s="1" t="s">
+        <v>770</v>
+      </c>
+      <c r="B247" s="1" t="s">
+        <v>750</v>
+      </c>
+      <c r="C247" s="1" t="s">
+        <v>759</v>
+      </c>
+      <c r="D247" s="1" t="s">
+        <v>771</v>
+      </c>
+      <c r="E247" s="2" t="s">
+        <v>825</v>
+      </c>
+      <c r="F247" s="2" t="s">
+        <v>826</v>
+      </c>
+      <c r="G247" s="1" t="s">
+        <v>827</v>
+      </c>
+    </row>
+    <row r="248" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A248" s="1" t="s">
+        <v>772</v>
+      </c>
+      <c r="B248" s="1" t="s">
+        <v>750</v>
+      </c>
+      <c r="C248" s="1" t="s">
+        <v>759</v>
+      </c>
+      <c r="D248" s="1" t="s">
+        <v>773</v>
+      </c>
+      <c r="E248" s="2" t="s">
         <v>846</v>
       </c>
-      <c r="F246" s="2" t="s">
+      <c r="F248" s="2" t="s">
         <v>847</v>
       </c>
-      <c r="G246" s="1" t="s">
-        <v>845</v>
-      </c>
-    </row>
-    <row r="247" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A247" s="1" t="s">
-        <v>772</v>
-      </c>
-      <c r="B247" s="1" t="s">
-        <v>752</v>
-      </c>
-      <c r="C247" s="1" t="s">
-        <v>761</v>
-      </c>
-      <c r="D247" s="1" t="s">
-        <v>773</v>
-      </c>
-      <c r="E247" s="2" t="s">
-        <v>827</v>
-      </c>
-      <c r="F247" s="2" t="s">
-        <v>828</v>
-      </c>
-      <c r="G247" s="1" t="s">
-        <v>829</v>
-      </c>
-    </row>
-    <row r="248" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A248" s="1" t="s">
+      <c r="G248" s="1" t="s">
+        <v>848</v>
+      </c>
+    </row>
+    <row r="249" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A249" s="1" t="s">
         <v>774</v>
       </c>
-      <c r="B248" s="1" t="s">
-        <v>752</v>
-      </c>
-      <c r="C248" s="1" t="s">
-        <v>761</v>
-      </c>
-      <c r="D248" s="1" t="s">
-        <v>775</v>
-      </c>
-      <c r="E248" s="2" t="s">
-        <v>848</v>
-      </c>
-      <c r="F248" s="2" t="s">
-        <v>849</v>
-      </c>
-      <c r="G248" s="1" t="s">
-        <v>850</v>
-      </c>
-    </row>
-    <row r="249" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A249" s="1" t="s">
-        <v>776</v>
-      </c>
       <c r="B249" s="1" t="s">
-        <v>752</v>
+        <v>750</v>
       </c>
       <c r="C249" s="1" t="s">
-        <v>761</v>
+        <v>759</v>
       </c>
       <c r="D249" s="1" t="s">
         <v>296</v>
       </c>
       <c r="E249" s="2" t="s">
-        <v>852</v>
+        <v>850</v>
       </c>
       <c r="F249" s="2" t="s">
-        <v>853</v>
+        <v>851</v>
       </c>
       <c r="G249" s="1" t="s">
-        <v>851</v>
-      </c>
-    </row>
-    <row r="250" spans="1:7" x14ac:dyDescent="0.35">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="250" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A250" s="1" t="s">
-        <v>777</v>
+        <v>775</v>
       </c>
       <c r="B250" s="1" t="s">
-        <v>752</v>
+        <v>750</v>
       </c>
       <c r="C250" s="1" t="s">
-        <v>761</v>
+        <v>759</v>
       </c>
       <c r="D250" s="1" t="s">
         <v>298</v>
       </c>
       <c r="E250" s="2" t="s">
-        <v>855</v>
+        <v>853</v>
       </c>
       <c r="F250" s="2" t="s">
-        <v>856</v>
+        <v>854</v>
       </c>
       <c r="G250" s="1" t="s">
-        <v>854</v>
-      </c>
-    </row>
-    <row r="251" spans="1:7" x14ac:dyDescent="0.35">
+        <v>852</v>
+      </c>
+    </row>
+    <row r="251" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A251" s="1" t="s">
+        <v>776</v>
+      </c>
+      <c r="B251" s="1" t="s">
+        <v>750</v>
+      </c>
+      <c r="C251" s="1" t="s">
+        <v>777</v>
+      </c>
+      <c r="D251" s="1" t="s">
+        <v>777</v>
+      </c>
+      <c r="E251" s="2" t="s">
         <v>778</v>
       </c>
-      <c r="B251" s="1" t="s">
-        <v>752</v>
-      </c>
-      <c r="C251" s="1" t="s">
+      <c r="F251" s="2" t="s">
         <v>779</v>
       </c>
-      <c r="D251" s="1" t="s">
-        <v>779</v>
-      </c>
-      <c r="E251" s="2" t="s">
+      <c r="G251" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="252" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A252" s="1" t="s">
         <v>780</v>
       </c>
-      <c r="F251" s="2" t="s">
+      <c r="B252" s="1" t="s">
+        <v>750</v>
+      </c>
+      <c r="C252" s="1" t="s">
         <v>781</v>
       </c>
-      <c r="G251" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="252" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A252" s="1" t="s">
+      <c r="D252" s="1" t="s">
+        <v>781</v>
+      </c>
+      <c r="E252" s="2" t="s">
         <v>782</v>
       </c>
-      <c r="B252" s="1" t="s">
-        <v>752</v>
-      </c>
-      <c r="C252" s="1" t="s">
+      <c r="F252" s="2" t="s">
         <v>783</v>
       </c>
-      <c r="D252" s="1" t="s">
-        <v>783</v>
-      </c>
-      <c r="E252" s="2" t="s">
+      <c r="G252" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="253" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A253" s="1" t="s">
         <v>784</v>
       </c>
-      <c r="F252" s="2" t="s">
+      <c r="B253" s="1" t="s">
+        <v>750</v>
+      </c>
+      <c r="C253" s="1" t="s">
         <v>785</v>
       </c>
-      <c r="G252" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="253" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A253" s="1" t="s">
+      <c r="D253" s="1" t="s">
+        <v>785</v>
+      </c>
+      <c r="E253" s="2" t="s">
         <v>786</v>
       </c>
-      <c r="B253" s="1" t="s">
-        <v>752</v>
-      </c>
-      <c r="C253" s="1" t="s">
+      <c r="F253" s="2" t="s">
         <v>787</v>
       </c>
-      <c r="D253" s="1" t="s">
-        <v>787</v>
-      </c>
-      <c r="E253" s="2" t="s">
+      <c r="G253" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="254" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A254" s="1" t="s">
         <v>788</v>
       </c>
-      <c r="F253" s="2" t="s">
+      <c r="B254" s="1" t="s">
+        <v>750</v>
+      </c>
+      <c r="C254" s="1" t="s">
         <v>789</v>
       </c>
-      <c r="G253" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="254" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A254" s="1" t="s">
-        <v>790</v>
-      </c>
-      <c r="B254" s="1" t="s">
-        <v>752</v>
-      </c>
-      <c r="C254" s="1" t="s">
-        <v>791</v>
-      </c>
       <c r="D254" s="1" t="s">
-        <v>791</v>
+        <v>789</v>
       </c>
       <c r="E254" s="2">
         <v>4.0039882000000002</v>
@@ -9413,113 +9607,113 @@
         <v>10</v>
       </c>
     </row>
-    <row r="255" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="255" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A255" s="1" t="s">
+        <v>790</v>
+      </c>
+      <c r="B255" s="1" t="s">
+        <v>750</v>
+      </c>
+      <c r="C255" s="1" t="s">
+        <v>791</v>
+      </c>
+      <c r="D255" s="1" t="s">
+        <v>791</v>
+      </c>
+      <c r="E255" s="2" t="s">
         <v>792</v>
       </c>
-      <c r="B255" s="1" t="s">
-        <v>752</v>
-      </c>
-      <c r="C255" s="1" t="s">
+      <c r="F255" s="2" t="s">
         <v>793</v>
       </c>
-      <c r="D255" s="1" t="s">
-        <v>793</v>
-      </c>
-      <c r="E255" s="2" t="s">
+      <c r="G255" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="256" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A256" s="1" t="s">
         <v>794</v>
       </c>
-      <c r="F255" s="2" t="s">
+      <c r="B256" s="1" t="s">
+        <v>750</v>
+      </c>
+      <c r="C256" s="1" t="s">
         <v>795</v>
       </c>
-      <c r="G255" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="256" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A256" s="1" t="s">
+      <c r="D256" s="1" t="s">
+        <v>795</v>
+      </c>
+      <c r="E256" s="2" t="s">
         <v>796</v>
       </c>
-      <c r="B256" s="1" t="s">
-        <v>752</v>
-      </c>
-      <c r="C256" s="1" t="s">
+      <c r="F256" s="2" t="s">
         <v>797</v>
       </c>
-      <c r="D256" s="1" t="s">
-        <v>797</v>
-      </c>
-      <c r="E256" s="2" t="s">
+      <c r="G256" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="257" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A257" s="1" t="s">
         <v>798</v>
       </c>
-      <c r="F256" s="2" t="s">
+      <c r="B257" s="1" t="s">
+        <v>750</v>
+      </c>
+      <c r="C257" s="1" t="s">
         <v>799</v>
       </c>
-      <c r="G256" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="257" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A257" s="1" t="s">
+      <c r="D257" s="1" t="s">
+        <v>799</v>
+      </c>
+      <c r="E257" s="2" t="s">
         <v>800</v>
       </c>
-      <c r="B257" s="1" t="s">
-        <v>752</v>
-      </c>
-      <c r="C257" s="1" t="s">
+      <c r="F257" s="2" t="s">
         <v>801</v>
       </c>
-      <c r="D257" s="1" t="s">
-        <v>801</v>
-      </c>
-      <c r="E257" s="2" t="s">
+      <c r="G257" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="258" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A258" s="1" t="s">
         <v>802</v>
       </c>
-      <c r="F257" s="2" t="s">
+      <c r="B258" s="1" t="s">
+        <v>750</v>
+      </c>
+      <c r="C258" s="1" t="s">
         <v>803</v>
       </c>
-      <c r="G257" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="258" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A258" s="1" t="s">
+      <c r="D258" s="1" t="s">
+        <v>803</v>
+      </c>
+      <c r="E258" s="2" t="s">
         <v>804</v>
       </c>
-      <c r="B258" s="1" t="s">
-        <v>752</v>
-      </c>
-      <c r="C258" s="1" t="s">
+      <c r="F258" s="2" t="s">
         <v>805</v>
       </c>
-      <c r="D258" s="1" t="s">
-        <v>805</v>
-      </c>
-      <c r="E258" s="2" t="s">
+      <c r="G258" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="259" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A259" s="1" t="s">
         <v>806</v>
       </c>
-      <c r="F258" s="2" t="s">
+      <c r="B259" s="1" t="s">
+        <v>750</v>
+      </c>
+      <c r="C259" s="1" t="s">
         <v>807</v>
       </c>
-      <c r="G258" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="259" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A259" s="1" t="s">
-        <v>808</v>
-      </c>
-      <c r="B259" s="1" t="s">
-        <v>752</v>
-      </c>
-      <c r="C259" s="1" t="s">
-        <v>809</v>
-      </c>
       <c r="D259" s="1" t="s">
-        <v>809</v>
+        <v>807</v>
       </c>
       <c r="E259" s="2" t="s">
-        <v>812</v>
+        <v>810</v>
       </c>
       <c r="F259" s="2">
         <v>-66.169397250800003</v>

</xml_diff>